<commit_message>
Updated Ecplise version to 2025 and Selenium to version 4 and made changes regarding waits
</commit_message>
<xml_diff>
--- a/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
+++ b/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhrx\git\repository\SeleniumAutomationFramework\src\test\resources\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D946619-9D50-47A0-BE9A-E0452F39E0EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED26485-74A8-420F-B6E8-3596F26FE7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{8729CB30-0DA3-4B54-AFF0-045232716AC7}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="57">
   <si>
     <t>testname</t>
   </si>
@@ -198,7 +198,16 @@
     <t>11</t>
   </si>
   <si>
-    <t>Orange Middle NameMiddle Name Test</t>
+    <t>test</t>
+  </si>
+  <si>
+    <t>verifThatTheAdminCanChangeUserInformation</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>verifyThatTheAdminCanChangeUserInformation</t>
   </si>
 </sst>
 </file>
@@ -557,10 +566,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C63E9A7D-678B-40CF-9D0A-F339110468CD}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="71.41796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.15625" customWidth="1"/>
     <col min="2" max="2" width="47.734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -765,6 +774,23 @@
         <v>52</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -775,7 +801,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A04EA249-C286-437E-A58A-69C4BA98E9D1}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="54.7890625" bestFit="1" customWidth="1"/>
@@ -912,6 +938,58 @@
         <v>49</v>
       </c>
       <c r="H5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added few changes regarding xpath
</commit_message>
<xml_diff>
--- a/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
+++ b/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhrx\git\repository\SeleniumAutomationFramework\src\test\resources\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp 2\OrangeHRM-Automation\SeleniumAutomationFramework\src\test\resources\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D946619-9D50-47A0-BE9A-E0452F39E0EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABC2388-8CC5-41E1-B35B-F8005CC6F3FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{8729CB30-0DA3-4B54-AFF0-045232716AC7}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="1" activeTab="1" xr2:uid="{8729CB30-0DA3-4B54-AFF0-045232716AC7}"/>
   </bookViews>
   <sheets>
     <sheet name="RUNMANAGER" sheetId="1" r:id="rId1"/>
@@ -18,19 +18,10 @@
     <sheet name="DATA" sheetId="2" r:id="rId3"/>
     <sheet name="USERACCOUNTMANAGEMENTDATA" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -198,7 +189,7 @@
     <t>11</t>
   </si>
   <si>
-    <t>Orange Middle NameMiddle Name Test</t>
+    <t>sww test</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changed employee name in exxcel file to john
</commit_message>
<xml_diff>
--- a/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
+++ b/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp 2\OrangeHRM-Automation\SeleniumAutomationFramework\src\test\resources\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABC2388-8CC5-41E1-B35B-F8005CC6F3FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6736586-8E1D-4A6A-89D1-D6124AD94DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" firstSheet="1" activeTab="1" xr2:uid="{8729CB30-0DA3-4B54-AFF0-045232716AC7}"/>
+    <workbookView xWindow="366" yWindow="366" windowWidth="17280" windowHeight="8088" firstSheet="1" activeTab="1" xr2:uid="{8729CB30-0DA3-4B54-AFF0-045232716AC7}"/>
   </bookViews>
   <sheets>
     <sheet name="RUNMANAGER" sheetId="1" r:id="rId1"/>
@@ -189,7 +189,7 @@
     <t>11</t>
   </si>
   <si>
-    <t>sww test</t>
+    <t>john</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added logger functionality to test and pages and listner class using log4j2
</commit_message>
<xml_diff>
--- a/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
+++ b/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp 2\OrangeHRM-Automation\SeleniumAutomationFramework\src\test\resources\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6736586-8E1D-4A6A-89D1-D6124AD94DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC14737-C445-40F0-8D94-B97CB1684BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="366" yWindow="366" windowWidth="17280" windowHeight="8088" firstSheet="1" activeTab="1" xr2:uid="{8729CB30-0DA3-4B54-AFF0-045232716AC7}"/>
   </bookViews>
@@ -189,7 +189,7 @@
     <t>11</t>
   </si>
   <si>
-    <t>john</t>
+    <t>j</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added logging functionality (#19)
* Fixed गलत merge conflict markers in RetryFailedTests

* Added logger functionality to test and pages and listner class using
log4j2
</commit_message>
<xml_diff>
--- a/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
+++ b/SeleniumAutomationFramework/src/test/resources/Excel/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp 2\OrangeHRM-Automation\SeleniumAutomationFramework\src\test\resources\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6736586-8E1D-4A6A-89D1-D6124AD94DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC14737-C445-40F0-8D94-B97CB1684BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="366" yWindow="366" windowWidth="17280" windowHeight="8088" firstSheet="1" activeTab="1" xr2:uid="{8729CB30-0DA3-4B54-AFF0-045232716AC7}"/>
   </bookViews>
@@ -189,7 +189,7 @@
     <t>11</t>
   </si>
   <si>
-    <t>john</t>
+    <t>j</t>
   </si>
 </sst>
 </file>

</xml_diff>